<commit_message>
actualizacion con casos de uso
</commit_message>
<xml_diff>
--- a/docs/planillas/Necesidades_Candidatas_PT.xlsx
+++ b/docs/planillas/Necesidades_Candidatas_PT.xlsx
@@ -1,19 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\sandbox-git\docs\planillas\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{095C858D-EF0B-4AFF-9299-58A0B165B77B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="51480" yWindow="-7380" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Perfiles Clientes" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Problema" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Necesidades" sheetId="3" r:id="rId7"/>
+    <sheet name="Perfiles Clientes" sheetId="1" r:id="rId1"/>
+    <sheet name="Problema" sheetId="2" r:id="rId2"/>
+    <sheet name="Necesidades" sheetId="3" r:id="rId3"/>
+    <sheet name="Necesidades Consolidadas" sheetId="4" r:id="rId4"/>
+    <sheet name="Casos de uso" sheetId="5" r:id="rId5"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="121">
   <si>
     <t>ID</t>
   </si>
@@ -126,15 +150,9 @@
     <t>Germán</t>
   </si>
   <si>
-    <t>Dificultad para medir de forma objetiva la percepción de esfuerzo de los atletas</t>
-  </si>
-  <si>
     <t>Gonzalo - Acta 003</t>
   </si>
   <si>
-    <t>*</t>
-  </si>
-  <si>
     <t>N4</t>
   </si>
   <si>
@@ -144,9 +162,6 @@
     <t>Registro/historial centralizado del alumno (síntesis transversal: presente en los 3 casos, con distinto énfasis)</t>
   </si>
   <si>
-    <t xml:space="preserve">Online </t>
-  </si>
-  <si>
     <t>Desfase leve entre el plan semanal de entrenamientos pactado y lo efectivamente ejecutado</t>
   </si>
   <si>
@@ -159,9 +174,6 @@
     <t>Candidata fuerte a necesidad principal del segmento PT</t>
   </si>
   <si>
-    <t>El propio entrevistado lo marca como problema menor</t>
-  </si>
-  <si>
     <t>C3</t>
   </si>
   <si>
@@ -180,42 +192,265 @@
     <t>Online y presencial</t>
   </si>
   <si>
-    <t>Planillas (rutina, seguimiento), formulario inicial, Drive (videos)</t>
-  </si>
-  <si>
     <t>P7</t>
   </si>
   <si>
-    <t>Videos de técnica dispersos en Drive, poco práctico de compartir</t>
-  </si>
-  <si>
     <t>P8</t>
   </si>
   <si>
     <t>Sin control estricto de pagos ni recordatorios automáticos a clientes</t>
+  </si>
+  <si>
+    <t>Excel compartido con el alumno (rutina, series, feedback de sensaciones/cargas); en modalidad presencial lo gestiona el PT, en modalidad online lo completa el propio alumno; WhatsApp para recibir videos de técnica; Loom para grabar feedback en video</t>
+  </si>
+  <si>
+    <t>P9</t>
+  </si>
+  <si>
+    <t>Sin registro de asistencia/clases tomadas por alumno; el seguimiento depende de la memoria del PT y del alumno</t>
+  </si>
+  <si>
+    <t>Gonzalo - Acta 003 / entrevista de seguimiento</t>
+  </si>
+  <si>
+    <t>Distinto del problema de pagos (P8), aunque relacionado: uno es "cuánto cobrar", este es "cuántas clases dio"</t>
+  </si>
+  <si>
+    <t>Impacto confirmado: "me ha pasado olvidarme si tal persona me pagó y tener que salir a revisar el chat de WhatsApp"</t>
+  </si>
+  <si>
+    <t>Videos de técnica dispersos en Drive; la barrera de acceso (buscar dentro de una carpeta compartida) dificulta que el alumno los use, no solo la dispersión en sí</t>
+  </si>
+  <si>
+    <t>N5</t>
+  </si>
+  <si>
+    <t>Contenido de entrenamiento (video + series/reps/programación) accesible en un solo lugar para el alumno, sin depender de buscar en una carpeta compartida</t>
+  </si>
+  <si>
+    <t>Gonzalo - entrevista de seguimiento</t>
+  </si>
+  <si>
+    <t>Relacionada con N3 (unificar todo), pero específica del contenido/video — considerar si se fusiona con N3 o queda separada</t>
+  </si>
+  <si>
+    <t>Evidencia relevante para 2.3: Gonzalo declara haber probado varias plataformas existentes antes de conformarse con su combinación actual de herramientas — "todas terminan siendo incompletas". Sirve para justificar por qué desarrollar una solución nueva en vez de adoptar una existente.</t>
+  </si>
+  <si>
+    <t>Mayormente online; corrige en persona a los alumnos que coinciden con su horario en sala/gimnasio</t>
+  </si>
+  <si>
+    <t>WhatsApp e Instagram para recibir videos de técnica del alumno; corrige en su horario laboral, no requiere envío inmediato</t>
+  </si>
+  <si>
+    <t>WhatsApp e Instagram</t>
+  </si>
+  <si>
+    <t>Necesita una forma de traducir la percepción subjetiva de esfuerzo del atleta (ej. "hoy me siento un 7 de cansado") en una prescripción objetiva de carga (peso y repeticiones concretas), en base a las marcas/PRs de ese atleta específico</t>
+  </si>
+  <si>
+    <t>Priorizado explícitamente por el propio Germán por sobre automatizar el envío del plan. Es más una funcionalidad de auto-regulación que un simple registro — evaluar si entra en el MVP o queda como mejora futura (a decidir en 2.13).</t>
+  </si>
+  <si>
+    <t>El plan de entrenamiento se actualiza semana a semana de forma manual vía WhatsApp, en base a cómo el atleta dice haberse sentido la semana anterior — un proceso que el propio PT describe como tedioso, ya que requiere estar pendiente todos los días. Su intención es avanzar hacia un cronograma más estructurado, pero hoy sigue siendo manual.</t>
+  </si>
+  <si>
+    <t>P10</t>
+  </si>
+  <si>
+    <t>Intentó sistematizar el registro con Excel, pero no tiene el manejo técnico necesario ("se me da para el culo") y abandonó el intento</t>
+  </si>
+  <si>
+    <t>Germán - entrevista larga</t>
+  </si>
+  <si>
+    <t>Relevante como requisito no funcional: la solución debe ser usable sin conocimientos técnicos/fórmulas, no asumir experticia en planillas</t>
+  </si>
+  <si>
+    <t>Necesidad</t>
+  </si>
+  <si>
+    <t>Basada en</t>
+  </si>
+  <si>
+    <t>NC1</t>
+  </si>
+  <si>
+    <t>Historial general del alumno: datos personales y evolución/progreso en el tiempo</t>
+  </si>
+  <si>
+    <t>N1, N2, N4</t>
+  </si>
+  <si>
+    <t>NC2</t>
+  </si>
+  <si>
+    <t>Historial médico del alumno: lesiones, restricciones físicas y estudios médicos</t>
+  </si>
+  <si>
+    <t>N1, P2</t>
+  </si>
+  <si>
+    <t>NC3</t>
+  </si>
+  <si>
+    <t>Contenido accesible en un solo lugar: rutina, videos de técnica y programación</t>
+  </si>
+  <si>
+    <t>N3, N5, P7</t>
+  </si>
+  <si>
+    <t>Registro de asistencia y pagos</t>
+  </si>
+  <si>
+    <t>NC4</t>
+  </si>
+  <si>
+    <t>P8, P9</t>
+  </si>
+  <si>
+    <t>NC5</t>
+  </si>
+  <si>
+    <t>Visibilidad de agenda</t>
+  </si>
+  <si>
+    <t>PRIORIDAD</t>
+  </si>
+  <si>
+    <t>Alta</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>NC6</t>
+  </si>
+  <si>
+    <t>Gestión de rutinas de entrenamiento: crear, asignar y ajustar rutinas (ejercicios, series, repeticiones, peso) para cada alumno</t>
+  </si>
+  <si>
+    <t>N2, P4, P5</t>
+  </si>
+  <si>
+    <t>list</t>
+  </si>
+  <si>
+    <t>NC0</t>
+  </si>
+  <si>
+    <t>Control de acceso: solo el PT y el alumno correspondiente pueden ver/editar su información</t>
+  </si>
+  <si>
+    <t>Justificada por la sensibilidad de datos médicos y de pagos que maneja el sistema</t>
+  </si>
+  <si>
+    <t>(transversal — no aplica)</t>
+  </si>
+  <si>
+    <t>Nombre del caso de uso</t>
+  </si>
+  <si>
+    <t>Necesidad (NC)</t>
+  </si>
+  <si>
+    <t>CU1</t>
+  </si>
+  <si>
+    <t>CU2</t>
+  </si>
+  <si>
+    <t>CU3</t>
+  </si>
+  <si>
+    <t>CU4</t>
+  </si>
+  <si>
+    <t>CU5</t>
+  </si>
+  <si>
+    <t>CU6</t>
+  </si>
+  <si>
+    <t>CU7</t>
+  </si>
+  <si>
+    <t>Registrar alumno</t>
+  </si>
+  <si>
+    <t>Editar datos del alumno</t>
+  </si>
+  <si>
+    <t>Marcar alumno como inactivo</t>
+  </si>
+  <si>
+    <t>Consultar historial del alumno</t>
+  </si>
+  <si>
+    <t>Iniciar sesión</t>
+  </si>
+  <si>
+    <t>Dar de alta a un alumno (genera su acceso)</t>
+  </si>
+  <si>
+    <t>Cerrar sesión</t>
+  </si>
+  <si>
+    <t>Transversal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	NC1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="14.0"/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -224,54 +459,52 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -461,27 +694,30 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="8.75"/>
-    <col customWidth="1" min="2" max="2" width="19.88"/>
-    <col customWidth="1" min="3" max="3" width="35.38"/>
-    <col customWidth="1" min="4" max="4" width="21.25"/>
-    <col customWidth="1" min="5" max="5" width="23.5"/>
-    <col customWidth="1" min="6" max="6" width="21.5"/>
-    <col customWidth="1" min="7" max="7" width="25.88"/>
-    <col customWidth="1" min="8" max="8" width="33.75"/>
+    <col min="1" max="1" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" customWidth="1"/>
+    <col min="3" max="3" width="35.42578125" customWidth="1"/>
+    <col min="4" max="4" width="21.28515625" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" customWidth="1"/>
+    <col min="6" max="6" width="21.42578125" customWidth="1"/>
+    <col min="7" max="7" width="68.85546875" customWidth="1"/>
+    <col min="8" max="8" width="33.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -506,105 +742,106 @@
       <c r="H1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" s="2"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" spans="1:9" ht="12.75">
+      <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="3">
-        <v>20.0</v>
-      </c>
-      <c r="E2" s="3">
-        <v>15.0</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="D2" s="2">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2">
+        <v>15</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:9" ht="12.75">
+      <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="D3" s="2">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="12.75">
+      <c r="A4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2">
+        <v>5</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>46</v>
-      </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="83.5"/>
-    <col customWidth="1" min="3" max="3" width="26.0"/>
-    <col customWidth="1" min="4" max="4" width="21.25"/>
-    <col customWidth="1" min="5" max="5" width="35.25"/>
+    <col min="2" max="2" width="202.7109375" customWidth="1"/>
+    <col min="3" max="3" width="35.85546875" customWidth="1"/>
+    <col min="4" max="4" width="21.28515625" customWidth="1"/>
+    <col min="5" max="5" width="35.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -620,150 +857,191 @@
       <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7" ht="12.75">
+      <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="D2" s="2">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:7" ht="12.75">
+      <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="s">
+      <c r="D3" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="12.75">
+      <c r="A4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="s">
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="12.75">
+      <c r="A5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="12.75">
+      <c r="A6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="12.75">
+      <c r="A7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="s">
+      <c r="D7" s="2">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="12.75">
+      <c r="A8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="12.75">
+      <c r="A9" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="E7" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="s">
+      <c r="C9" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C10" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="s">
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="3">
-        <v>1.0</v>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A11" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="3">
+        <v>1</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="9.63"/>
-    <col customWidth="1" min="2" max="2" width="86.38"/>
-    <col customWidth="1" min="3" max="3" width="36.5"/>
-    <col customWidth="1" min="4" max="4" width="22.38"/>
-    <col customWidth="1" min="5" max="5" width="44.75"/>
+    <col min="1" max="1" width="9.5703125" customWidth="1"/>
+    <col min="2" max="2" width="86.42578125" customWidth="1"/>
+    <col min="3" max="3" width="36.42578125" customWidth="1"/>
+    <col min="4" max="4" width="22.42578125" customWidth="1"/>
+    <col min="5" max="5" width="112.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -779,71 +1057,322 @@
       <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="2"/>
-    </row>
-    <row r="2">
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" ht="12.75">
+      <c r="A2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="12.75">
+      <c r="A3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="12.75">
+      <c r="A4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="12.75">
+      <c r="A5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="2">
+        <v>3</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76D88D74-B21E-475F-92E5-9AA2DDF77E10}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
+  <cols>
+    <col min="1" max="1" width="41.5703125" customWidth="1"/>
+    <col min="2" max="2" width="69.85546875" customWidth="1"/>
+    <col min="3" max="3" width="45" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="18">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>13</v>
+        <v>78</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>18</v>
+        <v>79</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>80</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="3" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>27</v>
+        <v>82</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D3" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>83</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="3" t="s">
-        <v>32</v>
+        <v>84</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>35</v>
+        <v>85</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D4" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>86</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="3" t="s">
-        <v>40</v>
+        <v>88</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D5" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>47</v>
+        <v>89</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F2D317C-C9BE-4275-B038-DBCC64DE3646}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
+  <cols>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="44.28515625" customWidth="1"/>
+    <col min="3" max="3" width="35.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="18">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
actualizacion casos de uso
</commit_message>
<xml_diff>
--- a/docs/planillas/Necesidades_Candidatas_PT.xlsx
+++ b/docs/planillas/Necesidades_Candidatas_PT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\sandbox-git\docs\planillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{095C858D-EF0B-4AFF-9299-58A0B165B77B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11D57319-973F-43E3-9CBC-43B3C7FBB054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51480" yWindow="-7380" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="146">
   <si>
     <t>ID</t>
   </si>
@@ -375,18 +375,6 @@
     <t>CU7</t>
   </si>
   <si>
-    <t>Registrar alumno</t>
-  </si>
-  <si>
-    <t>Editar datos del alumno</t>
-  </si>
-  <si>
-    <t>Marcar alumno como inactivo</t>
-  </si>
-  <si>
-    <t>Consultar historial del alumno</t>
-  </si>
-  <si>
     <t>Iniciar sesión</t>
   </si>
   <si>
@@ -399,14 +387,112 @@
     <t>Transversal</t>
   </si>
   <si>
-    <t xml:space="preserve">	NC1</t>
+    <t>Gestionar Alumno (CRUD)</t>
+  </si>
+  <si>
+    <t>Gestionar historial médico</t>
+  </si>
+  <si>
+    <t>NOTAS</t>
+  </si>
+  <si>
+    <r>
+      <t>Ver ficha del alumno</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (pantalla resumen: asistencia, médico, pagos, rutina)</t>
+    </r>
+  </si>
+  <si>
+    <t>ACTOR</t>
+  </si>
+  <si>
+    <t>PT</t>
+  </si>
+  <si>
+    <t>PT y Alumno</t>
+  </si>
+  <si>
+    <t>CU8</t>
+  </si>
+  <si>
+    <t>CU9</t>
+  </si>
+  <si>
+    <t>Gestionar agenda</t>
+  </si>
+  <si>
+    <t>CU10</t>
+  </si>
+  <si>
+    <t>Gestionar catálogo de ejercicios</t>
+  </si>
+  <si>
+    <t>Alumno</t>
+  </si>
+  <si>
+    <t>Interactuar con rutina asignada</t>
+  </si>
+  <si>
+    <t>Incluye: ver rutina (solo lectura), ver video de técnica de un ejercicio, y agregar nota — todo dentro de la misma pantalla/flujo</t>
+  </si>
+  <si>
+    <t>CU11</t>
+  </si>
+  <si>
+    <t>Armar y editar rutina de un alumno</t>
+  </si>
+  <si>
+    <t>Nombre, video asociado, contraindicaciones</t>
+  </si>
+  <si>
+    <t>Lesiones, comorbilidades, estudios</t>
+  </si>
+  <si>
+    <t>Pantalla resumen: asistencia, médico, pagos, rutina</t>
+  </si>
+  <si>
+    <t>CRUD de datos básicos</t>
+  </si>
+  <si>
+    <t>Drag &amp; drop; incluye validación de contraindicaciones al agregar un ejercicio</t>
+  </si>
+  <si>
+    <t>Ver disponibilidad, agendar/reagendar, recordatorio de cambio de horario, marcar asistencia de la sesión</t>
+  </si>
+  <si>
+    <t>Gestionar pagos</t>
+  </si>
+  <si>
+    <t>Incluye: registrar pago, recordatorio de vencimiento (ej. "estamos a 10"), generar comprobante/recibo, ver tendencia de pagos del alumno</t>
+  </si>
+  <si>
+    <t>Transversal + NC1</t>
+  </si>
+  <si>
+    <t>Solicita identificación, contacto y datos médicos (obligatorios); físicos, contexto y observaciones (opcionales). Genera el acceso del alumno.</t>
+  </si>
+  <si>
+    <t>CU12</t>
+  </si>
+  <si>
+    <t>Home del PT</t>
+  </si>
+  <si>
+    <t>Dashboard con resumen del día (sesiones agendadas, pagos pendientes) y accesos directos a alumnos, agenda, catálogo de ejercicios. Punto de entrada tras iniciar sesión</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -453,6 +539,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -474,7 +567,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -486,6 +579,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1276,15 +1370,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F2D317C-C9BE-4275-B038-DBCC64DE3646}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
-    <col min="2" max="2" width="44.28515625" customWidth="1"/>
+    <col min="2" max="2" width="79.140625" customWidth="1"/>
     <col min="3" max="3" width="35.7109375" customWidth="1"/>
+    <col min="4" max="4" width="69.5703125" customWidth="1"/>
+    <col min="5" max="5" width="43.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18">
+    <row r="1" spans="1:5" ht="18">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1294,8 +1390,14 @@
       <c r="C1" s="6" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
         <v>105</v>
       </c>
@@ -1303,73 +1405,194 @@
         <v>112</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>115</v>
+      </c>
+      <c r="D2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="B3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
         <v>107</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+        <v>113</v>
+      </c>
+      <c r="C4" t="s">
+        <v>141</v>
+      </c>
+      <c r="D4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" s="3" t="s">
         <v>108</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+        <v>78</v>
+      </c>
+      <c r="D5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="C6" s="3" t="s">
+      <c r="B6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" t="s">
+        <v>121</v>
+      </c>
+      <c r="E6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D7" t="s">
+        <v>121</v>
+      </c>
+      <c r="E7" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>119</v>
+      <c r="C8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D8" t="s">
+        <v>121</v>
+      </c>
+      <c r="E8" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B9" t="s">
+        <v>132</v>
+      </c>
+      <c r="C9" t="s">
+        <v>95</v>
+      </c>
+      <c r="D9" t="s">
+        <v>121</v>
+      </c>
+      <c r="E9" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>124</v>
+      </c>
+      <c r="B10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C10" t="s">
+        <v>84</v>
+      </c>
+      <c r="D10" t="s">
+        <v>128</v>
+      </c>
+      <c r="E10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" t="s">
+        <v>121</v>
+      </c>
+      <c r="E11" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>131</v>
+      </c>
+      <c r="B12" t="s">
+        <v>139</v>
+      </c>
+      <c r="C12" t="s">
+        <v>88</v>
+      </c>
+      <c r="D12" t="s">
+        <v>121</v>
+      </c>
+      <c r="E12" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>143</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D13" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>